<commit_message>
Prepare local-first deployment and release bundle
</commit_message>
<xml_diff>
--- a/maintenance/GenericLubrication_Maintenance_Tracker_Template.xlsx
+++ b/maintenance/GenericLubrication_Maintenance_Tracker_Template.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AS22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,24 +549,109 @@
           <t>Estimated duration min</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Last_Done_Draw</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Last_Done_Hours_UV1</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Last_Done_Hours_UV2</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Last_Done_Hours_Furnace</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Required_Tools</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Mandatory_Parts</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Conditional_Parts</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Preparation_Lead_Days</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Parts_Check_Lead_Days</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Auto_Order_Mandatory_Parts</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger_Modes</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger_Hours_Source</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger_Hours_Interval</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger_Draws_Interval</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger_Calendar_Value</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Trigger_Calendar_Unit</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Test_Preset</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Test_Fields</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Test_Thresholds</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Test_Condition</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Test_Action</t>
         </is>
       </c>
     </row>
@@ -609,6 +694,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>days</t>
@@ -640,11 +726,13 @@
           <t>Shielded/sealed-for-life bearings must NOT be lubricated.</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
         <v>0</v>
       </c>
@@ -664,6 +752,27 @@
       <c r="X2" t="n">
         <v>20</v>
       </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -704,6 +813,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>months</t>
@@ -735,11 +845,13 @@
           <t>Apply sparingly; remove excess oil.</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
         <v>0</v>
       </c>
@@ -759,6 +871,27 @@
       <c r="X3" t="n">
         <v>20</v>
       </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -799,6 +932,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>months</t>
@@ -830,11 +964,13 @@
           <t>Do not over-grease.</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>2026-02-04</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
         <v>0</v>
       </c>
@@ -854,6 +990,27 @@
       <c r="X4" t="n">
         <v>25</v>
       </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -894,6 +1051,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>months</t>
@@ -925,11 +1083,13 @@
           <t>Thin film only.</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
           <t>2025-09-29</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>0</v>
       </c>
@@ -949,6 +1109,27 @@
       <c r="X5" t="n">
         <v>25</v>
       </c>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -989,6 +1170,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>weeks</t>
@@ -1020,11 +1202,13 @@
           <t>Avoid oil contamination of fibre.</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
         <v>0</v>
       </c>
@@ -1044,6 +1228,27 @@
       <c r="X6" t="n">
         <v>25</v>
       </c>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1084,6 +1289,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>months</t>
@@ -1115,11 +1321,13 @@
           <t>Apply sparingly.</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
         <v>0</v>
       </c>
@@ -1139,6 +1347,27 @@
       <c r="X7" t="n">
         <v>25</v>
       </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1179,6 +1408,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>months</t>
@@ -1210,11 +1440,13 @@
           <t>Avoid oil migration into gas path.</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="n">
         <v>0</v>
       </c>
@@ -1234,6 +1466,27 @@
       <c r="X8" t="n">
         <v>25</v>
       </c>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1274,6 +1527,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>months</t>
@@ -1305,11 +1559,13 @@
           <t>Do not lubricate sealed bearings.</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
         <v>0</v>
       </c>
@@ -1329,6 +1585,27 @@
       <c r="X9" t="n">
         <v>25</v>
       </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1369,6 +1646,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>months</t>
@@ -1400,11 +1678,13 @@
           <t>Sealed-for-life bearings must not be lubricated.</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
         <v>0</v>
       </c>
@@ -1424,6 +1704,27 @@
       <c r="X10" t="n">
         <v>25</v>
       </c>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1464,6 +1765,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>months</t>
@@ -1495,11 +1797,13 @@
           <t>Remove surplus oil before operation.</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="n">
         <v>0</v>
       </c>
@@ -1519,6 +1823,27 @@
       <c r="X11" t="n">
         <v>25</v>
       </c>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1559,6 +1884,7 @@
           <t>calendar</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>months</t>
@@ -1590,11 +1916,13 @@
           <t>Do not over-grease.</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>2026-02-04</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
         <v>0</v>
       </c>
@@ -1614,6 +1942,1557 @@
       <c r="X12" t="n">
         <v>25</v>
       </c>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>G-MNT-001</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260517104033</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>FLOWP4033 Grease; FLOWP4033 Wipe</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W13" t="n">
+        <v>1</v>
+      </c>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>FLOWP4033 Wrench</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>FLOWP4033 Grease; FLOWP4033 Wipe</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>G-MNT-002</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528134355</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>FLOWP4355 Grease; FLOWP4355 Wipe</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W14" t="n">
+        <v>1</v>
+      </c>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>FLOWP4355 Wrench</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>FLOWP4355 Grease; FLOWP4355 Wipe</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>G-MNT-003</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528141555</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>FLOWP1555 Grease; FLOWP1555 Wipe</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W15" t="n">
+        <v>1</v>
+      </c>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>FLOWP1555 Wrench</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>FLOWP1555 Grease; FLOWP1555 Wipe</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr"/>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>G-MNT-004</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528142423</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>FLOWP2423 Grease; FLOWP2423 Wipe</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W16" t="n">
+        <v>1</v>
+      </c>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="n">
+        <v>163</v>
+      </c>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>FLOWP2423 Wrench</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>FLOWP2423 Grease; FLOWP2423 Wipe</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>G-MNT-005</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528142936</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>FLOWP2936 Grease; FLOWP2936 Wipe</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W17" t="n">
+        <v>1</v>
+      </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="n">
+        <v>164</v>
+      </c>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>FLOWP2936 Wrench</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>FLOWP2936 Grease; FLOWP2936 Wipe</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr"/>
+      <c r="AR17" t="inlineStr"/>
+      <c r="AS17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Full Flow Rig</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>FFR-MNT-001</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528144725</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>FLOWP4725 Grease; FLOWP4725 Wipe</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W18" t="n">
+        <v>1</v>
+      </c>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="n">
+        <v>165</v>
+      </c>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>FLOWP4725 Wrench</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>FLOWP4725 Grease; FLOWP4725 Wipe</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
+      <c r="AM18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Full Flow Rig</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FFR-MNT-002</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528150023</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>FLOWP0023 Grease; FLOWP0023 Wipe</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W19" t="n">
+        <v>1</v>
+      </c>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="n">
+        <v>166</v>
+      </c>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>FLOWP0023 Wrench</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>FLOWP0023 Grease; FLOWP0023 Wipe</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Full Flow Rig</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FFR-MNT-003</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528152016</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>FLOWP2016 Grease; FLOWP2016 Wipe</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W20" t="n">
+        <v>1</v>
+      </c>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="n">
+        <v>167</v>
+      </c>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>FLOWP2016 Wrench</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>FLOWP2016 Grease; FLOWP2016 Wipe</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr"/>
+      <c r="AL20" t="inlineStr"/>
+      <c r="AM20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr"/>
+      <c r="AQ20" t="inlineStr"/>
+      <c r="AR20" t="inlineStr"/>
+      <c r="AS20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Full Flow Rig</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>FFR-MNT-004</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528153013</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>FLOWP3013 Grease; FLOWP3013 Wipe</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W21" t="n">
+        <v>1</v>
+      </c>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="n">
+        <v>168</v>
+      </c>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>FLOWP3013 Wrench</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>FLOWP3013 Grease; FLOWP3013 Wipe</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI21" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Full Flow Rig</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FFR-MNT-005</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Weekly full flow 20260528154045</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Full flow smoke</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>weekly</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>General Maintenance Manual</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Run the weekly smoke maintenance task.</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Use PPE.</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>FLOWP4045 Grease; FLOWP4045 Wipe</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="W22" t="n">
+        <v>1</v>
+      </c>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="n">
+        <v>169</v>
+      </c>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>FLOWP4045 Wrench</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>FLOWP4045 Grease; FLOWP4045 Wipe</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>Calendar</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
+      <c r="AM22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Weeks</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr"/>
+      <c r="AQ22" t="inlineStr"/>
+      <c r="AR22" t="inlineStr"/>
+      <c r="AS22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>